<commit_message>
remove googledocs after dockerized share
</commit_message>
<xml_diff>
--- a/aio-platform/src/main/resources/ae/ac/cud/customs/alfresco_seed_user_data.xlsx
+++ b/aio-platform/src/main/resources/ae/ac/cud/customs/alfresco_seed_user_data.xlsx
@@ -1,17 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
-  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30228"/>
+  <workbookPr filterPrivacy="1"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F78F5E3E-6C99-43F3-83DB-B740FA8B9252}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="38280" yWindow="-120" windowWidth="38640" windowHeight="21840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
-    <sheet sheetId="1" name="Alfresco Seed Users" state="visible" r:id="rId4"/>
+    <sheet name="Alfresco Seed Users" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="68">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="28">
   <si>
     <t>firstName</t>
   </si>
@@ -37,15 +41,9 @@
     <t>telephone</t>
   </si>
   <si>
-    <t>John</t>
-  </si>
-  <si>
     <t>Doe</t>
   </si>
   <si>
-    <t>john.doe@example.com</t>
-  </si>
-  <si>
     <t>Test123!</t>
   </si>
   <si>
@@ -61,30 +59,18 @@
     <t>+1-555-0101</t>
   </si>
   <si>
-    <t>Jane</t>
-  </si>
-  <si>
     <t>Smith</t>
   </si>
   <si>
-    <t>jane.smith@example.com</t>
-  </si>
-  <si>
     <t>Developer</t>
   </si>
   <si>
     <t>+1-555-0102</t>
   </si>
   <si>
-    <t>Alice</t>
-  </si>
-  <si>
     <t>Johnson</t>
   </si>
   <si>
-    <t>alice.j@example.com</t>
-  </si>
-  <si>
     <t>Science Dept</t>
   </si>
   <si>
@@ -97,141 +83,41 @@
     <t>+1-555-0103</t>
   </si>
   <si>
-    <t>Bob</t>
-  </si>
-  <si>
-    <t>Williams</t>
-  </si>
-  <si>
-    <t>bob.w@example.com</t>
-  </si>
-  <si>
-    <t>Researcher</t>
-  </si>
-  <si>
-    <t>+1-555-0104</t>
-  </si>
-  <si>
-    <t>Charlie</t>
-  </si>
-  <si>
-    <t>Brown</t>
-  </si>
-  <si>
-    <t>charlie.b@example.com</t>
-  </si>
-  <si>
-    <t>Engineering Dept</t>
-  </si>
-  <si>
-    <t>Lecturer</t>
-  </si>
-  <si>
-    <t>Building C</t>
-  </si>
-  <si>
-    <t>+1-555-0105</t>
-  </si>
-  <si>
-    <t>Diana</t>
-  </si>
-  <si>
-    <t>Davis</t>
-  </si>
-  <si>
-    <t>diana.d@example.com</t>
-  </si>
-  <si>
-    <t>Lab Technician</t>
-  </si>
-  <si>
-    <t>+1-555-0106</t>
-  </si>
-  <si>
-    <t>Eve</t>
-  </si>
-  <si>
-    <t>Miller</t>
-  </si>
-  <si>
-    <t>eve.m@example.com</t>
-  </si>
-  <si>
-    <t>Arts Dept</t>
-  </si>
-  <si>
-    <t>Building D</t>
-  </si>
-  <si>
-    <t>+1-555-0107</t>
-  </si>
-  <si>
-    <t>Frank</t>
-  </si>
-  <si>
-    <t>Wilson</t>
-  </si>
-  <si>
-    <t>frank.w@example.com</t>
-  </si>
-  <si>
-    <t>Coordinator</t>
-  </si>
-  <si>
-    <t>+1-555-0108</t>
-  </si>
-  <si>
-    <t>Grace</t>
-  </si>
-  <si>
-    <t>Moore</t>
-  </si>
-  <si>
-    <t>grace.m@example.com</t>
-  </si>
-  <si>
-    <t>Admin</t>
-  </si>
-  <si>
-    <t>HR Manager</t>
-  </si>
-  <si>
-    <t>Main Office</t>
-  </si>
-  <si>
-    <t>+1-555-0109</t>
-  </si>
-  <si>
-    <t>Heidi</t>
-  </si>
-  <si>
-    <t>Taylor</t>
-  </si>
-  <si>
-    <t>heidi.t@example.com</t>
-  </si>
-  <si>
-    <t>Clerk</t>
-  </si>
-  <si>
-    <t>+1-555-0110</t>
+    <t>draft-john.doe@example.com</t>
+  </si>
+  <si>
+    <t>Draft John</t>
+  </si>
+  <si>
+    <t>Review Jane</t>
+  </si>
+  <si>
+    <t>review-jane.smith@example.com</t>
+  </si>
+  <si>
+    <t>Publish Alice</t>
+  </si>
+  <si>
+    <t>publish-alice.j@example.com</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="3" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-      <sz val="11"/>
-      <name val="Calibri"/>
     </font>
     <font>
       <b/>
+      <sz val="11"/>
       <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
     </font>
     <font>
       <sz val="11"/>
@@ -283,7 +169,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -294,6 +180,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -632,21 +519,21 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H11"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:H4"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="11" customWidth="1"/>
     <col min="2" max="2" width="10" customWidth="1"/>
-    <col min="3" max="3" width="24" customWidth="1"/>
+    <col min="3" max="3" width="34.6328125" customWidth="1"/>
     <col min="4" max="4" width="15" customWidth="1"/>
     <col min="5" max="5" width="18" customWidth="1"/>
     <col min="6" max="6" width="16" customWidth="1"/>
     <col min="7" max="8" width="13" customWidth="1"/>
-    <col min="9" max="24" width="13.571428571428571" customWidth="1"/>
+    <col min="9" max="24" width="13.54296875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -672,269 +559,87 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B2" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="C2" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="D2" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="E2" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="F2" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="G2" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="F2" s="2" t="s">
+      <c r="H2" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="G2" s="2" t="s">
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A3" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="B3" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="H2" s="2" t="s">
+      <c r="C3" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3" s="3" t="s">
         <v>15</v>
       </c>
+      <c r="G3" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="H3" s="3" t="s">
+        <v>16</v>
+      </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A3" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="B3" s="3" t="s">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A4" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="B4" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="C4" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E4" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="D3" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="E3" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="F3" s="3" t="s">
+      <c r="F4" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="G3" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="H3" s="3" t="s">
+      <c r="G4" s="2" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A4" s="2" t="s">
+      <c r="H4" s="2" t="s">
         <v>21</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="E4" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="F4" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="G4" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="H4" s="2" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A5" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="B5" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="E5" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="F5" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="G5" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="H5" s="3" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A6" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="E6" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="F6" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="G6" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="H6" s="2" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A7" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>41</v>
-      </c>
-      <c r="C7" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="D7" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="E7" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="F7" s="3" t="s">
-        <v>43</v>
-      </c>
-      <c r="G7" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="H7" s="3" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A8" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="D8" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="E8" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="F8" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="G8" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="H8" s="2" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A9" s="3" t="s">
-        <v>51</v>
-      </c>
-      <c r="B9" s="3" t="s">
-        <v>52</v>
-      </c>
-      <c r="C9" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="D9" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="E9" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="F9" s="3" t="s">
-        <v>54</v>
-      </c>
-      <c r="G9" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="H9" s="3" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A10" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="B10" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="C10" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="D10" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="E10" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="F10" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="G10" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="H10" s="2" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A11" s="3" t="s">
-        <v>63</v>
-      </c>
-      <c r="B11" s="3" t="s">
-        <v>64</v>
-      </c>
-      <c r="C11" s="3" t="s">
-        <v>65</v>
-      </c>
-      <c r="D11" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="E11" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="F11" s="3" t="s">
-        <v>66</v>
-      </c>
-      <c r="G11" s="3" t="s">
-        <v>61</v>
-      </c>
-      <c r="H11" s="3" t="s">
-        <v>67</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H11"/>
+  <autoFilter ref="A1:H4" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
</xml_diff>